<commit_message>
0259-2026: datos desde el expediente y R1 de prueba; fojas distingue escritos de parte y documentos de Indecopi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014QUd4VPDb7H3XTxZ25FgCr
</commit_message>
<xml_diff>
--- a/entrada/R1_DATOS.xlsx
+++ b/entrada/R1_DATOS.xlsx
@@ -620,11 +620,36 @@
           <t>0259-2026</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>901-2025/PS1</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Christian Erick García Chávez / Daniela Alvarado Arévalo</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>señor / señora</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>correo / correo</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>DTE / DTE2</t>
@@ -632,12 +657,12 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>11/12/2025</t>
+          <t>11/12/2025 / 11/12/2025</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Prellenado solo con lo que afirma el Excel de control; completar las columnas vacías.</t>
+          <t>Fuente: documentos del expediente (Documento de Elevación por Apelación N° 050-2026-PS1 del 16/09/2026; recurso firmado por Mesa de Partes el 11/12/2025 contra la Resolución Final Nº 2044-2025/PS1 del 14/11/2025). Un solo recurso de ambos denunciantes (abogado Rubén Antonio Reátegui Viena).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v1.1.0: 0259-2026, partes una por línea, fecha por expediente, cédula física = domicilio, Actions y Releases
- Encabezado con varias partes en líneas separadas (el verificador rechaza «/»).
- Columna FECHA_EMISION por expediente en R1_DATOS.
- Las cédulas del expediente mandan sobre el directorio: cédula física → domicilio.
- fojas.py separa escritos de parte de documentos de Indecopi, fecha de
  presentación por firma de Mesa de Partes, vías del expediente, _hojas/ para escaneados.
- Workflow: simulación y verificador en cada push; Release en cada etiqueta v*.
- README (última actualización), CHANGELOG y refutaciones 20-24.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014QUd4VPDb7H3XTxZ25FgCr
</commit_message>
<xml_diff>
--- a/entrada/R1_DATOS.xlsx
+++ b/entrada/R1_DATOS.xlsx
@@ -58,10 +58,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R24"/>
+  <dimension ref="A1:S24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,80 +444,85 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>FECHA_EMISION</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>FECHA_INGRESO_CC1</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>EXPEDIENTE_ORIGEN</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>DENUNCIANTE_NOMBRE</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DENUNCIANTE_TRATO</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>DENUNCIANTE_VIA</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>DENUNCIADOS_NOMBRES</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>DENUNCIADOS_VIAS</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>APELANTES</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>FECHAS_APELACION</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>RESOLUCION_APELADA</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>EXTREMO</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ESCRITOS</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>AUDIENCIA_FECHA</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>AUDIENCIA_HORA</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>AUDIENCIA_SOLICITUD</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>OBSERVACIONES</t>
         </is>
@@ -533,82 +539,87 @@
           <t>S1…S5 (vacío = se deduce)</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>DD/MM/AAAA solo si este expediente lleva fecha propia (vacío = la de la remesa)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>DD/MM/AAAA: fecha en que la CC1 recibió el expediente</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>vacío = el del Excel de control</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Como va en el texto, con tildes (varios: /)</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>señor / señora (varios: /)</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>correo / casilla / domicilio (vacío = correo)</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>vacío = razón social del directorio</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>correo / casilla / domicilio, en el orden de los denunciados (vacío = directorio)</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>DTE / DDO / DDO2 (dos: «DTE / DDO»)</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>DD/MM/AAAA, en el orden de APELANTES</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>«Resolución Final Nº 2157-2025/PS1» (S5: «Resolución 3 de fecha 11 de julio de 2025»)</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>opcional: «en el extremo que …»</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>escritos a trasladar distintos del recurso: «DTE 25/06/2026; DDO 19/12/2025»</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>S4: DD/MM/AAAA</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>S4: «16:00»</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>S4: «DDO 08/01/2026» (quién la pidió y fecha del escrito)</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>libre</t>
         </is>
@@ -627,42 +638,52 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>16/09/2026</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>901-2025/PS1</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Christian Erick García Chávez / Daniela Alvarado Arévalo</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>señor / señora</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>correo / correo</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
+          <t>domicilio</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t>DTE / DTE2</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>11/12/2025 / 11/12/2025</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Fuente: documentos del expediente (Documento de Elevación por Apelación N° 050-2026-PS1 del 16/09/2026; recurso firmado por Mesa de Partes el 11/12/2025 contra la Resolución Final Nº 2044-2025/PS1 del 14/11/2025). Un solo recurso de ambos denunciantes (abogado Rubén Antonio Reátegui Viena).</t>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Fuente: documentos del expediente (Documento de Elevación por Apelación N° 050-2026-PS1 del 16/09/2026; recurso firmado por Mesa de Partes el 11/12/2025 contra la Resolución Final Nº 2044-2025/PS1 del 14/11/2025). Un solo recurso de ambos denunciantes (abogado Rubén Antonio Reátegui Viena). Quálitas: domicilio, porque el expediente trae su cédula física con cargo (Av. Enrique Canaval y Moreyra 641, San Isidro; recibida el 20/11/2025). Fecha de emisión propia: 18/09/2026 (indicación del usuario).</t>
         </is>
       </c>
     </row>
@@ -672,17 +693,17 @@
           <t>0569-2026</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>0329-2026/PS1</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>DDO</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Prellenado solo con lo que afirma el Excel de control; completar las columnas vacías.</t>
         </is>
@@ -694,12 +715,12 @@
           <t>0606-2026</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>0506-2026/PS1</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>Prellenado solo con lo que afirma el Excel de control; completar las columnas vacías.</t>
         </is>
@@ -716,47 +737,47 @@
           <t>S1</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>31/07/2026</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>253-2026/PS1</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Francis Russell Sotelo Chavez</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>señor</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>casilla</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Rímac Seguros y Reaseguros S.A.</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>correo</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>DTE</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>CONTROL: datos tomados de la R1 ya revisada «1 608-2026-APE - RIMAC (Ad Hoc) - LSQok.docx» (corpus/r1).</t>
         </is>
@@ -768,12 +789,12 @@
           <t>0609-2026</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>1948-2025/PS1</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>Prellenado solo con lo que afirma el Excel de control; completar las columnas vacías.</t>
         </is>
@@ -790,47 +811,47 @@
           <t>S1</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>06/07/2026</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>2298-2025/PS1</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Joel Pilco Trinidad</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>señor</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>correo</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>Banco Interamericano de Finanzas S.A. / Chubb Perú S.A. Compañía de Seguros y Reaseguros</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>domicilio / casilla</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>DTE</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>CONTROL: datos tomados de la R1 ya revisada «R1 629-2026 - - LSQok.docx» (corpus/r1).</t>
         </is>
@@ -847,47 +868,47 @@
           <t>S1</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>10/07/2026</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>0010-2026/PS1</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Hernan Rodrigo Mar Perez</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>señor</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>correo</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>La Positiva Seguros y Reaseguros S.A.</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>casilla</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>DTE</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>CONTROL: datos tomados de la R1 ya revisada «R1 663-2026 - LSQok.docx» (corpus/r1).</t>
         </is>
@@ -904,47 +925,47 @@
           <t>S1</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>15/07/2026</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>0006-2026/PS1</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Jannett Isbel Alcantara Sanchez</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>señora</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>correo</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>La Positiva Seguros y Reaseguros S.A.</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>casilla</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>DTE</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>CONTROL: datos tomados de la R1 ya revisada «R1 685-2026 - LSQok.docx» (corpus/r1).</t>
         </is>
@@ -956,12 +977,12 @@
           <t>0607-2026</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>2042-20252/PS1</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="S11" t="inlineStr">
         <is>
           <t>Prellenado solo con lo que afirma el Excel de control; completar las columnas vacías.</t>
         </is>
@@ -978,47 +999,47 @@
           <t>S1</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>22/07/2026</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>0720-2026/PS1</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>José Luis Marcelo Lopez</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>señor</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>correo</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>Interseguro Compañia de Seguros S.A.</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>casilla</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>DTE</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="S12" t="inlineStr">
         <is>
           <t>PENDIENTE: la R1 del corpus («R1 726-2026 - tiene escrito adicional…») atribuye el recurso y un escrito del 05/09/2026 al «señor Carlos Andrés Gómez Ramos», que según el Excel es el abogado de Interseguro; la cédula confirma que el apelante es el señor José Luis Marcelo Lopez (apelación del 28/05/2026). Confirmar de quién es el escrito del 05/09/2026 (si es de Interseguro, el supuesto es S2) y la tilde del nombre (López).</t>
         </is>
@@ -1030,12 +1051,12 @@
           <t>0730-2026</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>0850-2026/PS1</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="S13" t="inlineStr">
         <is>
           <t>Prellenado solo con lo que afirma el Excel de control; completar las columnas vacías.</t>
         </is>
@@ -1052,52 +1073,52 @@
           <t>S1</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>22/07/2026</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>0546-2026/PS1</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Edith Rosario Hernandez Soriano</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>señora</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>correo</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>La Positiva Seguros y Reaseguros S.A. / Insurama Servicios Perú S.A.C.</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>correo / casilla</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>DTE</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>DTE 25/06/2026</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
+      <c r="S14" t="inlineStr">
         <is>
           <t>CONTROL: datos tomados de la R1 ya revisada «R1 731-2026 - LSQok.docx» (corpus/r1).</t>
         </is>
@@ -1114,47 +1135,47 @@
           <t>S1</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>22/07/2026</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>0420-2026/PS1</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Norma Lizeth Valderrama Nolasco</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>señora</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>correo</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>Quálitas Compañía de Seguros S.A</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>correo</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>DTE</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
+      <c r="S15" t="inlineStr">
         <is>
           <t>CONTROL: datos tomados de la R1 ya revisada «R1 733-2026 - LSQok.docx» (corpus/r1).</t>
         </is>
@@ -1171,47 +1192,47 @@
           <t>S1</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>30/07/2026</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>0426-2026/PS1</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>Jonathan Joel Gutierrez Zavaleta</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>señor</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>correo</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>Quálitas Compañía de Seguros S.A.</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>correo</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>DTE</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
+      <c r="S16" t="inlineStr">
         <is>
           <t>CONTROL: datos tomados de la R1 ya revisada «R1 742-2026 - LSQok.docx» (corpus/r1).</t>
         </is>
@@ -1223,12 +1244,12 @@
           <t>0771-2026</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>0352-2026/PS1</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="S17" t="inlineStr">
         <is>
           <t>Prellenado solo con lo que afirma el Excel de control; completar las columnas vacías.</t>
         </is>
@@ -1240,12 +1261,12 @@
           <t>0772-2026</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>0012-2026/PS1</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="S18" t="inlineStr">
         <is>
           <t>Prellenado solo con lo que afirma el Excel de control; completar las columnas vacías.</t>
         </is>
@@ -1257,12 +1278,12 @@
           <t>0773-2026</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>0815-2026/PS1</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="S19" t="inlineStr">
         <is>
           <t>Prellenado solo con lo que afirma el Excel de control; completar las columnas vacías.</t>
         </is>
@@ -1274,12 +1295,12 @@
           <t>0784-2026</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>0567-2026/PS1</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr">
+      <c r="S20" t="inlineStr">
         <is>
           <t>Prellenado solo con lo que afirma el Excel de control; completar las columnas vacías.</t>
         </is>
@@ -1291,12 +1312,12 @@
           <t>0790-2026</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>0696-2026/PS1</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr">
+      <c r="S21" t="inlineStr">
         <is>
           <t>Prellenado solo con lo que afirma el Excel de control; completar las columnas vacías.</t>
         </is>
@@ -1308,12 +1329,12 @@
           <t>0794-2026</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>0556-2026/PS1</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
+      <c r="S22" t="inlineStr">
         <is>
           <t>Prellenado solo con lo que afirma el Excel de control; completar las columnas vacías.</t>
         </is>
@@ -1325,12 +1346,12 @@
           <t>0806-2026</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>421-2025/PS1</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr">
+      <c r="S23" t="inlineStr">
         <is>
           <t>Prellenado solo con lo que afirma el Excel de control; completar las columnas vacías.</t>
         </is>
@@ -1342,12 +1363,12 @@
           <t>0807-2026</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>0178-2026/PS1</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
+      <c r="S24" t="inlineStr">
         <is>
           <t>Prellenado solo con lo que afirma el Excel de control; completar las columnas vacías.</t>
         </is>

</xml_diff>